<commit_message>
bullet points and ESCAPE abstract
</commit_message>
<xml_diff>
--- a/Raw data/lci-Abhi image SSP2-Base 2020 latest.xlsx
+++ b/Raw data/lci-Abhi image SSP2-Base 2020 latest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20401"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhinabera/Desktop/Prospective-LCA/Raw data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Prospective LCA\Raw data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{922CD3AB-BFAA-E94D-B7CD-64F4EE293C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2DB0FE-4745-4B31-B752-49F884610EAF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
+    <workbookView xWindow="0" yWindow="504" windowWidth="28800" windowHeight="17496" activeTab="2" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilities" sheetId="6" r:id="rId1"/>
@@ -28,10 +28,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1242,19 +1242,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E8D1F9-2651-4D58-AB8D-D63402B2F76A}">
   <dimension ref="A1:K310"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="70.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="70.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>45</v>
       </c>
@@ -1268,7 +1268,7 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -1278,7 +1278,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1292,7 +1292,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1306,7 +1306,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
@@ -1320,7 +1320,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
@@ -1334,7 +1334,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>6</v>
       </c>
@@ -1348,7 +1348,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>8</v>
       </c>
@@ -1362,7 +1362,7 @@
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1374,7 +1374,7 @@
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>11</v>
       </c>
@@ -1400,7 +1400,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -1424,7 +1424,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -1471,7 +1471,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="3"/>
@@ -1481,7 +1481,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1495,7 +1495,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>2</v>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>3</v>
       </c>
@@ -1523,7 +1523,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>5</v>
       </c>
@@ -1537,7 +1537,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>6</v>
       </c>
@@ -1551,7 +1551,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>8</v>
       </c>
@@ -1565,7 +1565,7 @@
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1577,7 +1577,7 @@
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>11</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>56</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>58</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>60</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>62</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>55</v>
       </c>
@@ -1720,7 +1720,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
@@ -1730,7 +1730,7 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -1744,7 +1744,7 @@
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>2</v>
       </c>
@@ -1758,7 +1758,7 @@
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>3</v>
       </c>
@@ -1772,7 +1772,7 @@
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>5</v>
       </c>
@@ -1786,7 +1786,7 @@
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>6</v>
       </c>
@@ -1800,7 +1800,7 @@
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>8</v>
       </c>
@@ -1814,7 +1814,7 @@
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1826,7 +1826,7 @@
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>11</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>63</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>65</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>67</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>69</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>55</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
@@ -1979,7 +1979,7 @@
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>0</v>
       </c>
@@ -1993,7 +1993,7 @@
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
         <v>2</v>
       </c>
@@ -2007,7 +2007,7 @@
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
         <v>3</v>
       </c>
@@ -2021,7 +2021,7 @@
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
         <v>5</v>
       </c>
@@ -2035,7 +2035,7 @@
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>6</v>
       </c>
@@ -2049,7 +2049,7 @@
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
         <v>8</v>
       </c>
@@ -2063,7 +2063,7 @@
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>10</v>
       </c>
@@ -2075,7 +2075,7 @@
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>11</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>71</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>53</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>73</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>62</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>55</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="3"/>
@@ -2228,7 +2228,7 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +2242,7 @@
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
         <v>2</v>
       </c>
@@ -2256,7 +2256,7 @@
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
         <v>3</v>
       </c>
@@ -2270,7 +2270,7 @@
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
         <v>5</v>
       </c>
@@ -2284,7 +2284,7 @@
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="8" t="s">
         <v>6</v>
       </c>
@@ -2298,7 +2298,7 @@
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="8" t="s">
         <v>8</v>
       </c>
@@ -2312,7 +2312,7 @@
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>10</v>
       </c>
@@ -2324,7 +2324,7 @@
       <c r="G63" s="8"/>
       <c r="H63" s="8"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="8" t="s">
         <v>11</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>77</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>62</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>55</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="3"/>
@@ -2454,7 +2454,7 @@
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>0</v>
       </c>
@@ -2468,7 +2468,7 @@
       <c r="G70" s="8"/>
       <c r="H70" s="8"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="8" t="s">
         <v>2</v>
       </c>
@@ -2482,7 +2482,7 @@
       <c r="G71" s="8"/>
       <c r="H71" s="8"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="8" t="s">
         <v>3</v>
       </c>
@@ -2496,7 +2496,7 @@
       <c r="G72" s="8"/>
       <c r="H72" s="8"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="8" t="s">
         <v>5</v>
       </c>
@@ -2510,7 +2510,7 @@
       <c r="G73" s="8"/>
       <c r="H73" s="8"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="8" t="s">
         <v>6</v>
       </c>
@@ -2524,7 +2524,7 @@
       <c r="G74" s="8"/>
       <c r="H74" s="8"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="8" t="s">
         <v>8</v>
       </c>
@@ -2538,7 +2538,7 @@
       <c r="G75" s="8"/>
       <c r="H75" s="8"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>10</v>
       </c>
@@ -2550,7 +2550,7 @@
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="8" t="s">
         <v>11</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>78</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>65</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>80</v>
       </c>
@@ -2648,7 +2648,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>62</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>55</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="3"/>
@@ -2704,7 +2704,7 @@
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>0</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="G84" s="8"/>
       <c r="H84" s="8"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="8" t="s">
         <v>2</v>
       </c>
@@ -2732,7 +2732,7 @@
       <c r="G85" s="8"/>
       <c r="H85" s="8"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="8" t="s">
         <v>3</v>
       </c>
@@ -2746,7 +2746,7 @@
       <c r="G86" s="8"/>
       <c r="H86" s="8"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="8" t="s">
         <v>5</v>
       </c>
@@ -2760,7 +2760,7 @@
       <c r="G87" s="8"/>
       <c r="H87" s="8"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="8" t="s">
         <v>6</v>
       </c>
@@ -2774,7 +2774,7 @@
       <c r="G88" s="8"/>
       <c r="H88" s="8"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="8" t="s">
         <v>8</v>
       </c>
@@ -2788,7 +2788,7 @@
       <c r="G89" s="8"/>
       <c r="H89" s="8"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>10</v>
       </c>
@@ -2800,7 +2800,7 @@
       <c r="G90" s="8"/>
       <c r="H90" s="8"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="8" t="s">
         <v>11</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>82</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>77</v>
       </c>
@@ -2874,7 +2874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>62</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>55</v>
       </c>
@@ -2920,7 +2920,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="3"/>
@@ -2930,7 +2930,7 @@
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>0</v>
       </c>
@@ -2944,7 +2944,7 @@
       <c r="G97" s="8"/>
       <c r="H97" s="8"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="8" t="s">
         <v>2</v>
       </c>
@@ -2958,7 +2958,7 @@
       <c r="G98" s="8"/>
       <c r="H98" s="8"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="8" t="s">
         <v>3</v>
       </c>
@@ -2972,7 +2972,7 @@
       <c r="G99" s="8"/>
       <c r="H99" s="8"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="8" t="s">
         <v>5</v>
       </c>
@@ -2986,7 +2986,7 @@
       <c r="G100" s="8"/>
       <c r="H100" s="8"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="8" t="s">
         <v>6</v>
       </c>
@@ -3000,7 +3000,7 @@
       <c r="G101" s="8"/>
       <c r="H101" s="8"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="8" t="s">
         <v>8</v>
       </c>
@@ -3014,7 +3014,7 @@
       <c r="G102" s="8"/>
       <c r="H102" s="8"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>10</v>
       </c>
@@ -3026,7 +3026,7 @@
       <c r="G103" s="8"/>
       <c r="H103" s="8"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="8" t="s">
         <v>11</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>170</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>51</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>56</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>63</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>71</v>
       </c>
@@ -3172,7 +3172,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>75</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>78</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>82</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="3"/>
@@ -3254,7 +3254,7 @@
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>0</v>
       </c>
@@ -3268,7 +3268,7 @@
       <c r="G114" s="8"/>
       <c r="H114" s="8"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="8" t="s">
         <v>2</v>
       </c>
@@ -3282,7 +3282,7 @@
       <c r="G115" s="8"/>
       <c r="H115" s="8"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="8" t="s">
         <v>3</v>
       </c>
@@ -3296,7 +3296,7 @@
       <c r="G116" s="8"/>
       <c r="H116" s="8"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="8" t="s">
         <v>5</v>
       </c>
@@ -3310,7 +3310,7 @@
       <c r="G117" s="8"/>
       <c r="H117" s="8"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="8" t="s">
         <v>6</v>
       </c>
@@ -3324,7 +3324,7 @@
       <c r="G118" s="8"/>
       <c r="H118" s="8"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="8" t="s">
         <v>8</v>
       </c>
@@ -3338,7 +3338,7 @@
       <c r="G119" s="8"/>
       <c r="H119" s="8"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>10</v>
       </c>
@@ -3350,7 +3350,7 @@
       <c r="G120" s="8"/>
       <c r="H120" s="8"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="8" t="s">
         <v>11</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>85</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>88</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>48</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>90</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>92</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>35</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>94</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>95</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="3"/>
@@ -3576,7 +3576,7 @@
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>0</v>
       </c>
@@ -3590,7 +3590,7 @@
       <c r="G131" s="8"/>
       <c r="H131" s="8"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="8" t="s">
         <v>2</v>
       </c>
@@ -3604,7 +3604,7 @@
       <c r="G132" s="8"/>
       <c r="H132" s="8"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133" s="8" t="s">
         <v>3</v>
       </c>
@@ -3618,7 +3618,7 @@
       <c r="G133" s="8"/>
       <c r="H133" s="8"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134" s="8" t="s">
         <v>5</v>
       </c>
@@ -3632,7 +3632,7 @@
       <c r="G134" s="8"/>
       <c r="H134" s="8"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135" s="8" t="s">
         <v>6</v>
       </c>
@@ -3646,7 +3646,7 @@
       <c r="G135" s="8"/>
       <c r="H135" s="8"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136" s="8" t="s">
         <v>8</v>
       </c>
@@ -3660,7 +3660,7 @@
       <c r="G136" s="8"/>
       <c r="H136" s="8"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>10</v>
       </c>
@@ -3672,7 +3672,7 @@
       <c r="G137" s="8"/>
       <c r="H137" s="8"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138" s="8" t="s">
         <v>11</v>
       </c>
@@ -3698,7 +3698,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>97</v>
       </c>
@@ -3722,7 +3722,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>100</v>
       </c>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="K140" s="14"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>37</v>
       </c>
@@ -3764,7 +3764,7 @@
       </c>
       <c r="K141" s="14"/>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>101</v>
       </c>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="K142" s="14"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>102</v>
       </c>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="K143" s="14"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>103</v>
       </c>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="K144" s="14"/>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>104</v>
       </c>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="K145" s="14"/>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>105</v>
       </c>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="K146" s="14"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>106</v>
       </c>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="K147" s="14"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>107</v>
       </c>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="K148" s="14"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>108</v>
       </c>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="K149" s="14"/>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>109</v>
       </c>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="K150" s="14"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>110</v>
       </c>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="K151" s="14"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>111</v>
       </c>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="K152" s="14"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>112</v>
       </c>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="K153" s="14"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>113</v>
       </c>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="K154" s="14"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>114</v>
       </c>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="K155" s="14"/>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>115</v>
       </c>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="K156" s="14"/>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>116</v>
       </c>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="K157" s="14"/>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>117</v>
       </c>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="K158" s="14"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>118</v>
       </c>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="K159" s="14"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="3"/>
@@ -4152,7 +4152,7 @@
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>0</v>
       </c>
@@ -4167,7 +4167,7 @@
       <c r="H161" s="8"/>
       <c r="I161" s="8"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A162" s="8" t="s">
         <v>2</v>
       </c>
@@ -4182,7 +4182,7 @@
       <c r="H162" s="8"/>
       <c r="I162" s="8"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A163" s="8" t="s">
         <v>3</v>
       </c>
@@ -4197,7 +4197,7 @@
       <c r="H163" s="8"/>
       <c r="I163" s="8"/>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A164" s="8" t="s">
         <v>5</v>
       </c>
@@ -4212,7 +4212,7 @@
       <c r="H164" s="8"/>
       <c r="I164" s="8"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A165" s="8" t="s">
         <v>6</v>
       </c>
@@ -4227,7 +4227,7 @@
       <c r="H165" s="8"/>
       <c r="I165" s="8"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A166" s="8" t="s">
         <v>8</v>
       </c>
@@ -4242,7 +4242,7 @@
       <c r="H166" s="8"/>
       <c r="I166" s="8"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>10</v>
       </c>
@@ -4255,7 +4255,7 @@
       <c r="H167" s="8"/>
       <c r="I167" s="8"/>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A168" s="8" t="s">
         <v>11</v>
       </c>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="I168" s="8"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A169" s="8" t="s">
         <v>29</v>
       </c>
@@ -4305,7 +4305,7 @@
       <c r="H169" s="8"/>
       <c r="I169" s="8"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A170" s="8" t="s">
         <v>124</v>
       </c>
@@ -4329,7 +4329,7 @@
       <c r="I170" s="8"/>
       <c r="K170" s="14"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A171" s="8" t="s">
         <v>127</v>
       </c>
@@ -4353,7 +4353,7 @@
       <c r="I171" s="8"/>
       <c r="K171" s="14"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A172" s="8" t="s">
         <v>129</v>
       </c>
@@ -4377,7 +4377,7 @@
       <c r="I172" s="8"/>
       <c r="K172" s="14"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A173" s="8" t="s">
         <v>131</v>
       </c>
@@ -4401,7 +4401,7 @@
       <c r="I173" s="8"/>
       <c r="K173" s="14"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A174" s="8" t="s">
         <v>122</v>
       </c>
@@ -4427,7 +4427,7 @@
       <c r="I174" s="8"/>
       <c r="K174" s="14"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A175" s="8" t="s">
         <v>132</v>
       </c>
@@ -4453,7 +4453,7 @@
       <c r="I175" s="8"/>
       <c r="K175" s="14"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A176" s="8" t="s">
         <v>134</v>
       </c>
@@ -4479,7 +4479,7 @@
       <c r="I176" s="8"/>
       <c r="K176" s="14"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A177" s="8" t="s">
         <v>136</v>
       </c>
@@ -4505,7 +4505,7 @@
       <c r="I177" s="8"/>
       <c r="K177" s="14"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A178" s="8" t="s">
         <v>138</v>
       </c>
@@ -4531,7 +4531,7 @@
       <c r="I178" s="8"/>
       <c r="K178" s="14"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A179" s="8" t="s">
         <v>139</v>
       </c>
@@ -4557,7 +4557,7 @@
       <c r="I179" s="8"/>
       <c r="K179" s="14"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A180" s="8" t="s">
         <v>140</v>
       </c>
@@ -4583,7 +4583,7 @@
       <c r="I180" s="8"/>
       <c r="K180" s="14"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A181" s="8" t="s">
         <v>143</v>
       </c>
@@ -4609,7 +4609,7 @@
       <c r="I181" s="8"/>
       <c r="K181" s="14"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A182" s="8" t="s">
         <v>146</v>
       </c>
@@ -4635,7 +4635,7 @@
       <c r="I182" s="8"/>
       <c r="K182" s="14"/>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A183" s="8" t="s">
         <v>148</v>
       </c>
@@ -4661,7 +4661,7 @@
       <c r="I183" s="8"/>
       <c r="K183" s="14"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A184" s="8" t="s">
         <v>150</v>
       </c>
@@ -4687,7 +4687,7 @@
       <c r="I184" s="8"/>
       <c r="K184" s="14"/>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A185" s="8" t="s">
         <v>152</v>
       </c>
@@ -4713,7 +4713,7 @@
       <c r="I185" s="8"/>
       <c r="K185" s="14"/>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A186" s="8" t="s">
         <v>154</v>
       </c>
@@ -4739,7 +4739,7 @@
       <c r="I186" s="8"/>
       <c r="K186" s="14"/>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -4750,7 +4750,7 @@
       <c r="H187" s="2"/>
       <c r="K187" s="14"/>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>0</v>
       </c>
@@ -4765,7 +4765,7 @@
       <c r="H188" s="8"/>
       <c r="K188" s="14"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A189" s="8" t="s">
         <v>2</v>
       </c>
@@ -4780,7 +4780,7 @@
       <c r="H189" s="8"/>
       <c r="K189" s="14"/>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A190" s="8" t="s">
         <v>3</v>
       </c>
@@ -4794,7 +4794,7 @@
       <c r="G190" s="8"/>
       <c r="H190" s="8"/>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A191" s="8" t="s">
         <v>5</v>
       </c>
@@ -4808,7 +4808,7 @@
       <c r="G191" s="8"/>
       <c r="H191" s="8"/>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A192" s="8" t="s">
         <v>6</v>
       </c>
@@ -4822,7 +4822,7 @@
       <c r="G192" s="8"/>
       <c r="H192" s="8"/>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A193" s="8" t="s">
         <v>8</v>
       </c>
@@ -4836,7 +4836,7 @@
       <c r="G193" s="8"/>
       <c r="H193" s="8"/>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>10</v>
       </c>
@@ -4848,7 +4848,7 @@
       <c r="G194" s="8"/>
       <c r="H194" s="8"/>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A195" s="8" t="s">
         <v>11</v>
       </c>
@@ -4874,7 +4874,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A196" s="8" t="s">
         <v>121</v>
       </c>
@@ -4898,7 +4898,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" s="8" t="s">
         <v>122</v>
       </c>
@@ -4922,7 +4922,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>55</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>29</v>
       </c>
@@ -4969,7 +4969,7 @@
       </c>
       <c r="H199" s="8"/>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -4979,7 +4979,7 @@
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>0</v>
       </c>
@@ -4993,7 +4993,7 @@
       <c r="G201" s="8"/>
       <c r="H201" s="8"/>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A202" s="8" t="s">
         <v>2</v>
       </c>
@@ -5007,7 +5007,7 @@
       <c r="G202" s="8"/>
       <c r="H202" s="8"/>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A203" s="8" t="s">
         <v>3</v>
       </c>
@@ -5021,7 +5021,7 @@
       <c r="G203" s="8"/>
       <c r="H203" s="8"/>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A204" s="8" t="s">
         <v>5</v>
       </c>
@@ -5035,7 +5035,7 @@
       <c r="G204" s="8"/>
       <c r="H204" s="8"/>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A205" s="8" t="s">
         <v>6</v>
       </c>
@@ -5049,7 +5049,7 @@
       <c r="G205" s="8"/>
       <c r="H205" s="8"/>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A206" s="8" t="s">
         <v>8</v>
       </c>
@@ -5063,7 +5063,7 @@
       <c r="G206" s="8"/>
       <c r="H206" s="8"/>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A207" s="1" t="s">
         <v>10</v>
       </c>
@@ -5075,7 +5075,7 @@
       <c r="G207" s="8"/>
       <c r="H207" s="8"/>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A208" s="8" t="s">
         <v>11</v>
       </c>
@@ -5101,7 +5101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A209" s="8" t="s">
         <v>158</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A210" s="8" t="s">
         <v>122</v>
       </c>
@@ -5149,7 +5149,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>55</v>
       </c>
@@ -5173,7 +5173,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>29</v>
       </c>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="H212" s="8"/>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -5206,7 +5206,7 @@
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A214" s="1" t="s">
         <v>0</v>
       </c>
@@ -5220,7 +5220,7 @@
       <c r="G214" s="8"/>
       <c r="H214" s="8"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A215" s="8" t="s">
         <v>2</v>
       </c>
@@ -5234,7 +5234,7 @@
       <c r="G215" s="8"/>
       <c r="H215" s="8"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A216" s="8" t="s">
         <v>3</v>
       </c>
@@ -5248,7 +5248,7 @@
       <c r="G216" s="8"/>
       <c r="H216" s="8"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A217" s="8" t="s">
         <v>5</v>
       </c>
@@ -5262,7 +5262,7 @@
       <c r="G217" s="8"/>
       <c r="H217" s="8"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A218" s="8" t="s">
         <v>6</v>
       </c>
@@ -5276,7 +5276,7 @@
       <c r="G218" s="8"/>
       <c r="H218" s="8"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A219" s="8" t="s">
         <v>8</v>
       </c>
@@ -5290,7 +5290,7 @@
       <c r="G219" s="8"/>
       <c r="H219" s="8"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A220" s="1" t="s">
         <v>10</v>
       </c>
@@ -5302,7 +5302,7 @@
       <c r="G220" s="8"/>
       <c r="H220" s="8"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A221" s="8" t="s">
         <v>11</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A222" s="8" t="s">
         <v>161</v>
       </c>
@@ -5352,7 +5352,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>85</v>
       </c>
@@ -5376,7 +5376,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A224" s="8" t="s">
         <v>158</v>
       </c>
@@ -5400,7 +5400,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A225" s="8" t="s">
         <v>163</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A226" s="8" t="s">
         <v>159</v>
       </c>
@@ -5448,7 +5448,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>29</v>
       </c>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="H227" s="8"/>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A228" s="2"/>
       <c r="B228" s="2"/>
       <c r="C228" s="3"/>
@@ -5480,7 +5480,7 @@
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A229" s="1" t="s">
         <v>0</v>
       </c>
@@ -5494,7 +5494,7 @@
       <c r="G229" s="8"/>
       <c r="H229" s="8"/>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A230" s="8" t="s">
         <v>2</v>
       </c>
@@ -5508,7 +5508,7 @@
       <c r="G230" s="8"/>
       <c r="H230" s="8"/>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A231" s="8" t="s">
         <v>3</v>
       </c>
@@ -5522,7 +5522,7 @@
       <c r="G231" s="8"/>
       <c r="H231" s="8"/>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A232" s="8" t="s">
         <v>5</v>
       </c>
@@ -5536,7 +5536,7 @@
       <c r="G232" s="8"/>
       <c r="H232" s="8"/>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A233" s="8" t="s">
         <v>6</v>
       </c>
@@ -5550,7 +5550,7 @@
       <c r="G233" s="8"/>
       <c r="H233" s="8"/>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A234" s="8" t="s">
         <v>8</v>
       </c>
@@ -5564,7 +5564,7 @@
       <c r="G234" s="8"/>
       <c r="H234" s="8"/>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A235" s="1" t="s">
         <v>10</v>
       </c>
@@ -5576,7 +5576,7 @@
       <c r="G235" s="8"/>
       <c r="H235" s="8"/>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A236" s="8" t="s">
         <v>11</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A237" s="8" t="s">
         <v>159</v>
       </c>
@@ -5626,7 +5626,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>85</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A239" s="8" t="s">
         <v>158</v>
       </c>
@@ -5674,7 +5674,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>55</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A241" s="8" t="s">
         <v>161</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>29</v>
       </c>
@@ -5743,7 +5743,7 @@
       </c>
       <c r="H242" s="8"/>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A243" s="2"/>
       <c r="B243" s="2"/>
       <c r="C243" s="3"/>
@@ -5753,7 +5753,7 @@
       <c r="G243" s="2"/>
       <c r="H243" s="2"/>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A244" s="1" t="s">
         <v>0</v>
       </c>
@@ -5767,7 +5767,7 @@
       <c r="G244" s="8"/>
       <c r="H244" s="8"/>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A245" s="8" t="s">
         <v>2</v>
       </c>
@@ -5781,7 +5781,7 @@
       <c r="G245" s="8"/>
       <c r="H245" s="8"/>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A246" s="8" t="s">
         <v>3</v>
       </c>
@@ -5795,7 +5795,7 @@
       <c r="G246" s="8"/>
       <c r="H246" s="8"/>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A247" s="8" t="s">
         <v>5</v>
       </c>
@@ -5809,7 +5809,7 @@
       <c r="G247" s="8"/>
       <c r="H247" s="8"/>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A248" s="8" t="s">
         <v>6</v>
       </c>
@@ -5823,7 +5823,7 @@
       <c r="G248" s="8"/>
       <c r="H248" s="8"/>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A249" s="8" t="s">
         <v>8</v>
       </c>
@@ -5837,7 +5837,7 @@
       <c r="G249" s="8"/>
       <c r="H249" s="8"/>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A250" s="1" t="s">
         <v>10</v>
       </c>
@@ -5849,7 +5849,7 @@
       <c r="G250" s="8"/>
       <c r="H250" s="8"/>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A251" s="8" t="s">
         <v>11</v>
       </c>
@@ -5875,7 +5875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A252" s="8" t="s">
         <v>40</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A253" s="5" t="s">
         <v>168</v>
       </c>
@@ -5923,7 +5923,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A254" s="7" t="s">
         <v>32</v>
       </c>
@@ -5945,7 +5945,7 @@
       </c>
       <c r="H254" s="8"/>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A255" s="5" t="s">
         <v>38</v>
       </c>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="H255" s="8"/>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A256" s="2"/>
       <c r="B256" s="2"/>
       <c r="C256" s="3"/>
@@ -5978,7 +5978,7 @@
       <c r="G256" s="2"/>
       <c r="H256" s="2"/>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A257" s="19" t="s">
         <v>0</v>
       </c>
@@ -5992,7 +5992,7 @@
       <c r="G257" s="5"/>
       <c r="H257" s="5"/>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A258" s="19" t="s">
         <v>2</v>
       </c>
@@ -6006,7 +6006,7 @@
       <c r="G258" s="5"/>
       <c r="H258" s="5"/>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A259" s="19" t="s">
         <v>3</v>
       </c>
@@ -6020,7 +6020,7 @@
       <c r="G259" s="5"/>
       <c r="H259" s="5"/>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A260" s="1" t="s">
         <v>6</v>
       </c>
@@ -6034,7 +6034,7 @@
       <c r="G260" s="5"/>
       <c r="H260" s="5"/>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A261" s="19" t="s">
         <v>5</v>
       </c>
@@ -6048,7 +6048,7 @@
       <c r="G261" s="5"/>
       <c r="H261" s="5"/>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A262" s="19" t="s">
         <v>8</v>
       </c>
@@ -6062,7 +6062,7 @@
       <c r="G262" s="5"/>
       <c r="H262" s="5"/>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A263" s="19" t="s">
         <v>201</v>
       </c>
@@ -6074,7 +6074,7 @@
       <c r="G263" s="5"/>
       <c r="H263" s="5"/>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A264" s="19" t="s">
         <v>10</v>
       </c>
@@ -6086,7 +6086,7 @@
       <c r="G264" s="5"/>
       <c r="H264" s="5"/>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A265" s="5" t="s">
         <v>11</v>
       </c>
@@ -6112,7 +6112,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A266" s="17" t="s">
         <v>185</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>47</v>
       </c>
@@ -6160,7 +6160,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A268" s="17" t="s">
         <v>202</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A269" s="17" t="s">
         <v>204</v>
       </c>
@@ -6208,7 +6208,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A270" s="17" t="s">
         <v>206</v>
       </c>
@@ -6232,7 +6232,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>29</v>
       </c>
@@ -6253,7 +6253,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>101</v>
       </c>
@@ -6274,7 +6274,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>100</v>
       </c>
@@ -6295,7 +6295,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274" s="18" t="s">
         <v>207</v>
       </c>
@@ -6316,7 +6316,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>37</v>
       </c>
@@ -6337,7 +6337,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276" s="18" t="s">
         <v>195</v>
       </c>
@@ -6358,7 +6358,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277" s="18" t="s">
         <v>105</v>
       </c>
@@ -6379,7 +6379,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278" s="18" t="s">
         <v>208</v>
       </c>
@@ -6400,7 +6400,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279" s="18" t="s">
         <v>209</v>
       </c>
@@ -6421,7 +6421,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280" s="18" t="s">
         <v>210</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281" s="18" t="s">
         <v>115</v>
       </c>
@@ -6463,7 +6463,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282" s="18" t="s">
         <v>211</v>
       </c>
@@ -6484,7 +6484,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283" s="18" t="s">
         <v>212</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284" s="18" t="s">
         <v>196</v>
       </c>
@@ -6524,7 +6524,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285" s="18" t="s">
         <v>108</v>
       </c>
@@ -6544,7 +6544,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A286" s="18" t="s">
         <v>213</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A287" s="18" t="s">
         <v>214</v>
       </c>
@@ -6584,7 +6584,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A288" s="18" t="s">
         <v>215</v>
       </c>
@@ -6604,7 +6604,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A289" s="18" t="s">
         <v>216</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A290" s="18" t="s">
         <v>217</v>
       </c>
@@ -6644,7 +6644,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="291" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A291" s="2"/>
       <c r="B291" s="2"/>
       <c r="C291" s="3"/>
@@ -6654,7 +6654,7 @@
       <c r="G291" s="2"/>
       <c r="H291" s="2"/>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A292" s="19" t="s">
         <v>0</v>
       </c>
@@ -6668,7 +6668,7 @@
       <c r="G292" s="5"/>
       <c r="H292" s="5"/>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A293" s="19" t="s">
         <v>2</v>
       </c>
@@ -6682,7 +6682,7 @@
       <c r="G293" s="5"/>
       <c r="H293" s="5"/>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A294" s="19" t="s">
         <v>3</v>
       </c>
@@ -6696,7 +6696,7 @@
       <c r="G294" s="5"/>
       <c r="H294" s="5"/>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A295" s="1" t="s">
         <v>6</v>
       </c>
@@ -6710,7 +6710,7 @@
       <c r="G295" s="5"/>
       <c r="H295" s="5"/>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A296" s="19" t="s">
         <v>5</v>
       </c>
@@ -6724,7 +6724,7 @@
       <c r="G296" s="5"/>
       <c r="H296" s="5"/>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A297" s="19" t="s">
         <v>8</v>
       </c>
@@ -6738,7 +6738,7 @@
       <c r="G297" s="5"/>
       <c r="H297" s="5"/>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A298" s="19" t="s">
         <v>10</v>
       </c>
@@ -6750,7 +6750,7 @@
       <c r="G298" s="5"/>
       <c r="H298" s="5"/>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A299" s="5" t="s">
         <v>11</v>
       </c>
@@ -6776,7 +6776,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A300" s="17" t="s">
         <v>206</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>55</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="302" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>225</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="303" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>227</v>
       </c>
@@ -6870,7 +6870,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>229</v>
       </c>
@@ -6893,7 +6893,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>231</v>
       </c>
@@ -6916,7 +6916,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>233</v>
       </c>
@@ -6939,7 +6939,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>88</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="308" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>235</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="309" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>90</v>
       </c>
@@ -7008,7 +7008,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>95</v>
       </c>
@@ -7040,17 +7040,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD968991-55C9-4627-9323-29F50518FFEB}">
   <dimension ref="A1:H80"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="86.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7064,7 +7064,7 @@
       <c r="G1" s="8"/>
       <c r="H1" s="8"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -7078,7 +7078,7 @@
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
@@ -7092,7 +7092,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
@@ -7106,7 +7106,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>6</v>
       </c>
@@ -7120,7 +7120,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
@@ -7134,7 +7134,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -7146,7 +7146,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>11</v>
       </c>
@@ -7172,7 +7172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -7196,7 +7196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -7244,7 +7244,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -7267,7 +7267,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>180</v>
       </c>
@@ -7291,7 +7291,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>239</v>
       </c>
@@ -7314,7 +7314,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>240</v>
       </c>
@@ -7338,7 +7338,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>242</v>
       </c>
@@ -7384,7 +7384,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -7404,7 +7404,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -7424,7 +7424,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -7445,7 +7445,7 @@
       </c>
       <c r="H20" s="14"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -7466,7 +7466,7 @@
       </c>
       <c r="H21" s="14"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -7486,7 +7486,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -7506,7 +7506,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="3"/>
@@ -7516,7 +7516,7 @@
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>0</v>
       </c>
@@ -7530,7 +7530,7 @@
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>2</v>
       </c>
@@ -7544,7 +7544,7 @@
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>3</v>
       </c>
@@ -7558,7 +7558,7 @@
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>5</v>
       </c>
@@ -7572,7 +7572,7 @@
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>6</v>
       </c>
@@ -7586,7 +7586,7 @@
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>8</v>
       </c>
@@ -7600,7 +7600,7 @@
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
@@ -7612,7 +7612,7 @@
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>11</v>
       </c>
@@ -7638,7 +7638,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>165</v>
       </c>
@@ -7662,7 +7662,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>47</v>
       </c>
@@ -7686,7 +7686,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
         <v>185</v>
       </c>
@@ -7710,7 +7710,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>55</v>
       </c>
@@ -7733,7 +7733,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>180</v>
       </c>
@@ -7757,7 +7757,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>239</v>
       </c>
@@ -7780,7 +7780,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>240</v>
       </c>
@@ -7804,7 +7804,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -7827,7 +7827,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
         <v>242</v>
       </c>
@@ -7850,7 +7850,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>37</v>
       </c>
@@ -7870,7 +7870,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>38</v>
       </c>
@@ -7890,7 +7890,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>36</v>
       </c>
@@ -7911,7 +7911,7 @@
       </c>
       <c r="H44" s="14"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>29</v>
       </c>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="H45" s="14"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>38</v>
       </c>
@@ -7952,7 +7952,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -7972,7 +7972,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="3"/>
@@ -7982,7 +7982,7 @@
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>0</v>
       </c>
@@ -7996,7 +7996,7 @@
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>2</v>
       </c>
@@ -8010,7 +8010,7 @@
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>3</v>
       </c>
@@ -8024,7 +8024,7 @@
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
         <v>5</v>
       </c>
@@ -8038,7 +8038,7 @@
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="8" t="s">
         <v>6</v>
       </c>
@@ -8052,7 +8052,7 @@
       <c r="G53" s="8"/>
       <c r="H53" s="8"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
         <v>8</v>
       </c>
@@ -8066,7 +8066,7 @@
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>10</v>
       </c>
@@ -8078,7 +8078,7 @@
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
         <v>11</v>
       </c>
@@ -8104,7 +8104,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>171</v>
       </c>
@@ -8128,7 +8128,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
         <v>40</v>
       </c>
@@ -8152,7 +8152,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>78</v>
       </c>
@@ -8176,7 +8176,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>27</v>
       </c>
@@ -8200,7 +8200,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>32</v>
       </c>
@@ -8220,7 +8220,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>55</v>
       </c>
@@ -8243,7 +8243,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>34</v>
       </c>
@@ -8263,7 +8263,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>35</v>
       </c>
@@ -8283,7 +8283,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>37</v>
       </c>
@@ -8303,7 +8303,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>38</v>
       </c>
@@ -8324,7 +8324,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>38</v>
       </c>
@@ -8345,7 +8345,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
         <v>154</v>
       </c>
@@ -8368,40 +8368,40 @@
         <v>155</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B69" s="15"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B70" s="15"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B71" s="15"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B72" s="15"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B73" s="4"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B74" s="15"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B75" s="15"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B76" s="15"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B77" s="15"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B78" s="15"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B79" s="15"/>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="8"/>
       <c r="B80" s="13"/>
       <c r="C80" s="8"/>
@@ -8419,17 +8419,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20D067F8-C305-44D3-8E28-CF1FDCAD7A72}">
   <dimension ref="A1:H75"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="86.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="33.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8443,7 +8443,7 @@
       <c r="G1" s="8"/>
       <c r="H1" s="8"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -8457,7 +8457,7 @@
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
@@ -8471,7 +8471,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>5</v>
       </c>
@@ -8485,7 +8485,7 @@
       <c r="G4" s="8"/>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>6</v>
       </c>
@@ -8499,7 +8499,7 @@
       <c r="G5" s="8"/>
       <c r="H5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
@@ -8513,7 +8513,7 @@
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -8525,7 +8525,7 @@
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>11</v>
       </c>
@@ -8551,7 +8551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>172</v>
       </c>
@@ -8575,7 +8575,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -8599,7 +8599,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -8646,7 +8646,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>176</v>
       </c>
@@ -8670,7 +8670,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>178</v>
       </c>
@@ -8694,7 +8694,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -8718,7 +8718,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>180</v>
       </c>
@@ -8742,7 +8742,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -8766,7 +8766,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>181</v>
       </c>
@@ -8791,7 +8791,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>182</v>
       </c>
@@ -8814,7 +8814,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>100</v>
       </c>
@@ -8834,7 +8834,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -8854,7 +8854,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>188</v>
       </c>
@@ -8874,7 +8874,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -8894,7 +8894,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -8914,7 +8914,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>189</v>
       </c>
@@ -8934,7 +8934,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>190</v>
       </c>
@@ -8954,7 +8954,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>191</v>
       </c>
@@ -8974,7 +8974,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>192</v>
       </c>
@@ -8994,7 +8994,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>190</v>
       </c>
@@ -9014,7 +9014,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -9034,7 +9034,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>193</v>
       </c>
@@ -9054,7 +9054,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>194</v>
       </c>
@@ -9074,7 +9074,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>195</v>
       </c>
@@ -9094,7 +9094,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>196</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>197</v>
       </c>
@@ -9134,7 +9134,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
         <v>198</v>
       </c>
@@ -9155,7 +9155,7 @@
       </c>
       <c r="H36" s="8"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
         <v>199</v>
       </c>
@@ -9177,7 +9177,7 @@
       </c>
       <c r="H37" s="8"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="3"/>
@@ -9187,7 +9187,7 @@
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>0</v>
       </c>
@@ -9201,7 +9201,7 @@
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
         <v>2</v>
       </c>
@@ -9215,7 +9215,7 @@
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>3</v>
       </c>
@@ -9229,7 +9229,7 @@
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
         <v>5</v>
       </c>
@@ -9243,7 +9243,7 @@
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
         <v>6</v>
       </c>
@@ -9257,7 +9257,7 @@
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
         <v>8</v>
       </c>
@@ -9271,7 +9271,7 @@
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>10</v>
       </c>
@@ -9283,7 +9283,7 @@
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
         <v>11</v>
       </c>
@@ -9309,7 +9309,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>175</v>
       </c>
@@ -9333,7 +9333,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -9357,7 +9357,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="17" t="s">
         <v>185</v>
       </c>
@@ -9381,7 +9381,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -9404,7 +9404,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>176</v>
       </c>
@@ -9428,7 +9428,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>178</v>
       </c>
@@ -9452,7 +9452,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>73</v>
       </c>
@@ -9476,7 +9476,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>180</v>
       </c>
@@ -9500,7 +9500,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>49</v>
       </c>
@@ -9524,7 +9524,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>181</v>
       </c>
@@ -9549,7 +9549,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>182</v>
       </c>
@@ -9572,7 +9572,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>100</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -9612,7 +9612,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>188</v>
       </c>
@@ -9632,7 +9632,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>37</v>
       </c>
@@ -9652,7 +9652,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>38</v>
       </c>
@@ -9672,7 +9672,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>189</v>
       </c>
@@ -9692,7 +9692,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>190</v>
       </c>
@@ -9712,7 +9712,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>191</v>
       </c>
@@ -9732,7 +9732,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>192</v>
       </c>
@@ -9752,7 +9752,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>190</v>
       </c>
@@ -9772,7 +9772,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>38</v>
       </c>
@@ -9792,7 +9792,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>193</v>
       </c>
@@ -9812,7 +9812,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>194</v>
       </c>
@@ -9832,7 +9832,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>195</v>
       </c>
@@ -9852,7 +9852,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>196</v>
       </c>
@@ -9872,7 +9872,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>197</v>
       </c>
@@ -9892,7 +9892,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="8" t="s">
         <v>198</v>
       </c>
@@ -9913,7 +9913,7 @@
       </c>
       <c r="H74" s="8"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="8" t="s">
         <v>199</v>
       </c>
@@ -9944,18 +9944,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{998EBEEB-B02A-47FC-B25F-8D09BAB943A0}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9963,7 +9963,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -9971,7 +9971,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -9979,7 +9979,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -9987,7 +9987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -9995,7 +9995,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -10003,12 +10003,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -10034,7 +10034,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>224</v>
       </c>
@@ -10057,7 +10057,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>172</v>
       </c>
@@ -10080,7 +10080,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -10104,7 +10104,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -10126,7 +10126,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>221</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>88</v>
       </c>
@@ -10172,7 +10172,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -10192,7 +10192,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -10212,7 +10212,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>223</v>
       </c>
@@ -10235,7 +10235,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>94</v>
       </c>

</xml_diff>

<commit_message>
correctiong in heating inventories
</commit_message>
<xml_diff>
--- a/Raw data/lci-Abhi image SSP2-Base 2020 latest.xlsx
+++ b/Raw data/lci-Abhi image SSP2-Base 2020 latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhinabera/Desktop/Prospective-LCA/Raw data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47F7E86-A444-DC40-83A7-6F3A803B014F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898B220A-02E7-2246-9448-E531F38A62D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilities" sheetId="6" r:id="rId1"/>
@@ -3162,8 +3162,8 @@
         <v>133</v>
       </c>
       <c r="B124" s="9">
-        <f>0.00116842105263158+0.146*B126/0.1*0.9</f>
-        <v>8.9140568526315783E-3</v>
+        <f>0.00116842105263158</f>
+        <v>1.1684210526315801E-3</v>
       </c>
       <c r="C124" t="s">
         <v>18</v>

</xml_diff>